<commit_message>
Notebook 03: one beat per cell, every sheet shown in context with the change shaded
170 cells, 72 of them code, each under the sentence that announces it: every lever is
give / do / check, and the refusals sit in the check where the prose puts them. A lever
writes into the workbook and then draws the sheet as it stands, the rows already there
for context and the rows just written shaded, with the file's own row numbers; an edit
draws the same window before and after. The example workbook and the one the levers
build are drawn as sheets, and the factor targets in the shape of the sheets that hold
them. All 23 readings rewritten from this run, including the shape claim, which is
within two tenths and not within Monte Carlo error: a third moment of a fat-tailed
asset moves by 0.16 across seeds.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/inputs/template.xlsx
+++ b/examples/inputs/template.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="20">
   <si>
     <t>ticker</t>
   </si>
@@ -37,6 +37,27 @@
   </si>
   <si>
     <t>kurt</t>
+  </si>
+  <si>
+    <t>Equity DM</t>
+  </si>
+  <si>
+    <t>Equity EM</t>
+  </si>
+  <si>
+    <t>Real premia</t>
+  </si>
+  <si>
+    <t>Inflation</t>
+  </si>
+  <si>
+    <t>Credit</t>
+  </si>
+  <si>
+    <t>Commodity</t>
+  </si>
+  <si>
+    <t>Small cap</t>
   </si>
   <si>
     <t>factor</t>
@@ -445,12 +466,33 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:1">
+    <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
         <v>1</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -468,13 +510,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -489,13 +531,13 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -510,7 +552,7 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>2</v>
@@ -537,13 +579,13 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>